<commit_message>
Keel stops earning Distribution Rewards from August 2026 (and Sky keeps the $1,531) (#193)
Co-authored-by: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/keel/2026-08/keel_settlement_august_2026.xlsx
+++ b/settlements/keel/2026-08/keel_settlement_august_2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Debt" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -501,37 +501,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>+ distribution_rewards (settle-dr-dune)</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>1530.91</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" s="4" t="n">
-        <v>33306.68174154446</v>
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" s="4" t="n">
+        <v>31775.77174154446</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sky side</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Sky side</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CoF on utilized (BR × Net_Subs)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CoF on utilized (BR × Net_Subs)</t>
+          <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -539,37 +539,37 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" s="4" t="n">
-        <v>0</v>
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Comparison (Grove-style "Profit to Grove")</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Comparison (Grove-style "Profit to Grove")</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>prime_agent_revenue</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>prime_agent_revenue</t>
+          <t>− CoF (deducted per-venue in display)</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
@@ -577,64 +577,54 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>− CoF (deducted per-venue in display)</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" s="4" t="n">
-        <v>0</v>
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-08-01 → 2026-08-31 (31 days)</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Pin blocks</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-01 → 2026-08-31 (31 days)</t>
+          <t>ethereum=25878704</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pin blocks</t>
+          <t>Generated</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ethereum=25878704</t>
+          <t>2026-09-02T22:05:20+00:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
-        <is>
-          <t>2026-09-01T14:41:44+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>

</xml_diff>